<commit_message>
Atualização na pagina dashboard, implementação de novos cards
</commit_message>
<xml_diff>
--- a/public/templates/importacao/03_clientes.xlsx
+++ b/public/templates/importacao/03_clientes.xlsx
@@ -397,13 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,6 +423,9 @@
       <c r="E1" t="str">
         <v>status</v>
       </c>
+      <c r="F1" t="str">
+        <v>e_rede</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -439,13 +443,16 @@
       <c r="E2" t="str">
         <v>Ativo</v>
       </c>
+      <c r="F2" t="str">
+        <v>Não</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>5002</v>
       </c>
       <c r="B3" t="str">
-        <v>Distribuidora São José LTDA</v>
+        <v>Rede Distribuidora São José</v>
       </c>
       <c r="C3" t="str">
         <v>98.765.432/0001-10</v>
@@ -455,11 +462,14 @@
       </c>
       <c r="E3" t="str">
         <v>Ativo</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Sim</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>